<commit_message>
feat: add TC6 Contact Us with file upload and alert handling
</commit_message>
<xml_diff>
--- a/Data Files/register_data.xlsx
+++ b/Data Files/register_data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/muhamadanangmahrub/Documents/katalon-projects/Automation_Exercise/Data Files/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0A8115D1-9928-804E-B466-59202B75E85E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{026B477E-28C8-AF49-846B-CBB50EBD1097}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="380" yWindow="500" windowWidth="28040" windowHeight="16300" xr2:uid="{46A2D747-70A5-2849-BFFB-98A89757B1C8}"/>
+    <workbookView xWindow="380" yWindow="500" windowWidth="28040" windowHeight="16280" xr2:uid="{46A2D747-70A5-2849-BFFB-98A89757B1C8}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -574,8 +574,7 @@
     <col min="8" max="8" width="8.83203125" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="15" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="17.6640625" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="9" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="12.33203125" bestFit="1" customWidth="1"/>
+    <col min="12" max="13" width="12.33203125" bestFit="1" customWidth="1"/>
     <col min="14" max="14" width="10.1640625" bestFit="1" customWidth="1"/>
     <col min="15" max="15" width="7.33203125" bestFit="1" customWidth="1"/>
     <col min="16" max="16" width="13.1640625" style="3" bestFit="1" customWidth="1"/>

</xml_diff>

<commit_message>
feat: add TC12 and refactor CartPage with dynamic parameterization
</commit_message>
<xml_diff>
--- a/Data Files/register_data.xlsx
+++ b/Data Files/register_data.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10510"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10517"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/muhamadanangmahrub/Documents/katalon-projects/Automation_Exercise/Data Files/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{026B477E-28C8-AF49-846B-CBB50EBD1097}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9934A9DA-9665-DE47-88C8-25D1F904F140}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="380" yWindow="500" windowWidth="28040" windowHeight="16280" xr2:uid="{46A2D747-70A5-2849-BFFB-98A89757B1C8}"/>
+    <workbookView xWindow="380" yWindow="500" windowWidth="28040" windowHeight="16140" xr2:uid="{46A2D747-70A5-2849-BFFB-98A89757B1C8}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -118,9 +118,6 @@
     <t>Siti Rahma</t>
   </si>
   <si>
-    <t>siti.rahma@example.com</t>
-  </si>
-  <si>
     <t>SitiSecure!45</t>
   </si>
   <si>
@@ -145,9 +142,6 @@
     <t>Budi Santoso</t>
   </si>
   <si>
-    <t>budi.santoso@example.com</t>
-  </si>
-  <si>
     <t>BudiPass@789</t>
   </si>
   <si>
@@ -188,6 +182,12 @@
   </si>
   <si>
     <t>Singapore</t>
+  </si>
+  <si>
+    <t>siti.rahma13@example.com</t>
+  </si>
+  <si>
+    <t>budi.santoso13@example.com</t>
   </si>
 </sst>
 </file>
@@ -665,7 +665,7 @@
         <v>23</v>
       </c>
       <c r="L2" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="M2" t="s">
         <v>24</v>
@@ -677,7 +677,7 @@
         <v>55213</v>
       </c>
       <c r="P2" s="3" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
     </row>
     <row r="3" spans="1:16" x14ac:dyDescent="0.2">
@@ -685,10 +685,10 @@
         <v>26</v>
       </c>
       <c r="B3" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="C3" t="s">
         <v>27</v>
-      </c>
-      <c r="C3" t="s">
-        <v>28</v>
       </c>
       <c r="D3">
         <v>27</v>
@@ -700,45 +700,45 @@
         <v>1995</v>
       </c>
       <c r="G3" t="s">
+        <v>28</v>
+      </c>
+      <c r="H3" t="s">
         <v>29</v>
       </c>
-      <c r="H3" t="s">
+      <c r="I3" t="s">
         <v>30</v>
       </c>
-      <c r="I3" t="s">
+      <c r="J3" t="s">
         <v>31</v>
       </c>
-      <c r="J3" t="s">
+      <c r="K3" t="s">
         <v>32</v>
       </c>
-      <c r="K3" t="s">
-        <v>33</v>
-      </c>
       <c r="L3" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="M3" t="s">
         <v>24</v>
       </c>
       <c r="N3" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="O3">
         <v>55581</v>
       </c>
       <c r="P3" s="3" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
     </row>
     <row r="4" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
+        <v>34</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="C4" t="s">
         <v>35</v>
-      </c>
-      <c r="B4" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="C4" t="s">
-        <v>37</v>
       </c>
       <c r="D4">
         <v>3</v>
@@ -750,41 +750,41 @@
         <v>2000</v>
       </c>
       <c r="G4" t="s">
+        <v>36</v>
+      </c>
+      <c r="H4" t="s">
+        <v>37</v>
+      </c>
+      <c r="I4" t="s">
         <v>38</v>
       </c>
-      <c r="H4" t="s">
+      <c r="J4" t="s">
         <v>39</v>
       </c>
-      <c r="I4" t="s">
+      <c r="K4" t="s">
         <v>40</v>
       </c>
-      <c r="J4" t="s">
+      <c r="L4" t="s">
+        <v>48</v>
+      </c>
+      <c r="M4" t="s">
         <v>41</v>
       </c>
-      <c r="K4" t="s">
+      <c r="N4" t="s">
         <v>42</v>
-      </c>
-      <c r="L4" t="s">
-        <v>50</v>
-      </c>
-      <c r="M4" t="s">
-        <v>43</v>
-      </c>
-      <c r="N4" t="s">
-        <v>44</v>
       </c>
       <c r="O4">
         <v>57411</v>
       </c>
       <c r="P4" s="3" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="B2" r:id="rId1" display="mailto:ahmad.fauzi@example.com" xr:uid="{4B90666F-B4DC-1D40-B23F-4994EB5457AC}"/>
-    <hyperlink ref="B3" r:id="rId2" display="mailto:siti.rahma@example.com" xr:uid="{287C8E49-AD8F-6F42-A67A-401A81B9FCFC}"/>
-    <hyperlink ref="B4" r:id="rId3" display="mailto:budi.santoso@example.com" xr:uid="{5999E4BB-BE5E-A141-AB26-57D4AE28AF3D}"/>
+    <hyperlink ref="B3" r:id="rId2" xr:uid="{287C8E49-AD8F-6F42-A67A-401A81B9FCFC}"/>
+    <hyperlink ref="B4" r:id="rId3" xr:uid="{5999E4BB-BE5E-A141-AB26-57D4AE28AF3D}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
feat: implement advance testing
- Add BrowserExecutionListener
- fix headless mode timing with implicit wait
</commit_message>
<xml_diff>
--- a/Data Files/register_data.xlsx
+++ b/Data Files/register_data.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10517"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10628"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/muhamadanangmahrub/Documents/katalon-projects/Automation_Exercise/Data Files/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9934A9DA-9665-DE47-88C8-25D1F904F140}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BEED9260-F4F2-D24E-9B23-BF86B2AFB5A7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="380" yWindow="500" windowWidth="28040" windowHeight="16140" xr2:uid="{46A2D747-70A5-2849-BFFB-98A89757B1C8}"/>
   </bookViews>
@@ -88,9 +88,6 @@
     <t>Ahmad Fauzi</t>
   </si>
   <si>
-    <t>ahmad.fauzi@example.com</t>
-  </si>
-  <si>
     <t>Ahmad#2026</t>
   </si>
   <si>
@@ -184,10 +181,13 @@
     <t>Singapore</t>
   </si>
   <si>
-    <t>siti.rahma13@example.com</t>
-  </si>
-  <si>
-    <t>budi.santoso13@example.com</t>
+    <t>ahmad.fauzi23@example.com</t>
+  </si>
+  <si>
+    <t>siti.rahma23@example.com</t>
+  </si>
+  <si>
+    <t>budi.santoso23@example.com</t>
   </si>
 </sst>
 </file>
@@ -635,10 +635,10 @@
         <v>16</v>
       </c>
       <c r="B2" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="C2" t="s">
         <v>17</v>
-      </c>
-      <c r="C2" t="s">
-        <v>18</v>
       </c>
       <c r="D2">
         <v>12</v>
@@ -650,45 +650,45 @@
         <v>1998</v>
       </c>
       <c r="G2" t="s">
+        <v>18</v>
+      </c>
+      <c r="H2" t="s">
         <v>19</v>
       </c>
-      <c r="H2" t="s">
+      <c r="I2" t="s">
         <v>20</v>
       </c>
-      <c r="I2" t="s">
+      <c r="J2" t="s">
         <v>21</v>
       </c>
-      <c r="J2" t="s">
+      <c r="K2" t="s">
         <v>22</v>
       </c>
-      <c r="K2" t="s">
+      <c r="L2" t="s">
+        <v>45</v>
+      </c>
+      <c r="M2" t="s">
         <v>23</v>
       </c>
-      <c r="L2" t="s">
-        <v>46</v>
-      </c>
-      <c r="M2" t="s">
+      <c r="N2" t="s">
         <v>24</v>
-      </c>
-      <c r="N2" t="s">
-        <v>25</v>
       </c>
       <c r="O2">
         <v>55213</v>
       </c>
       <c r="P2" s="3" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="3" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B3" s="2" t="s">
         <v>49</v>
       </c>
       <c r="C3" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="D3">
         <v>27</v>
@@ -700,45 +700,45 @@
         <v>1995</v>
       </c>
       <c r="G3" t="s">
+        <v>27</v>
+      </c>
+      <c r="H3" t="s">
         <v>28</v>
       </c>
-      <c r="H3" t="s">
+      <c r="I3" t="s">
         <v>29</v>
       </c>
-      <c r="I3" t="s">
+      <c r="J3" t="s">
         <v>30</v>
       </c>
-      <c r="J3" t="s">
+      <c r="K3" t="s">
         <v>31</v>
       </c>
-      <c r="K3" t="s">
+      <c r="L3" t="s">
+        <v>46</v>
+      </c>
+      <c r="M3" t="s">
+        <v>23</v>
+      </c>
+      <c r="N3" t="s">
         <v>32</v>
-      </c>
-      <c r="L3" t="s">
-        <v>47</v>
-      </c>
-      <c r="M3" t="s">
-        <v>24</v>
-      </c>
-      <c r="N3" t="s">
-        <v>33</v>
       </c>
       <c r="O3">
         <v>55581</v>
       </c>
       <c r="P3" s="3" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
     </row>
     <row r="4" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B4" s="2" t="s">
         <v>50</v>
       </c>
       <c r="C4" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="D4">
         <v>3</v>
@@ -750,39 +750,39 @@
         <v>2000</v>
       </c>
       <c r="G4" t="s">
+        <v>35</v>
+      </c>
+      <c r="H4" t="s">
         <v>36</v>
       </c>
-      <c r="H4" t="s">
+      <c r="I4" t="s">
         <v>37</v>
       </c>
-      <c r="I4" t="s">
+      <c r="J4" t="s">
         <v>38</v>
       </c>
-      <c r="J4" t="s">
+      <c r="K4" t="s">
         <v>39</v>
       </c>
-      <c r="K4" t="s">
+      <c r="L4" t="s">
+        <v>47</v>
+      </c>
+      <c r="M4" t="s">
         <v>40</v>
       </c>
-      <c r="L4" t="s">
-        <v>48</v>
-      </c>
-      <c r="M4" t="s">
+      <c r="N4" t="s">
         <v>41</v>
-      </c>
-      <c r="N4" t="s">
-        <v>42</v>
       </c>
       <c r="O4">
         <v>57411</v>
       </c>
       <c r="P4" s="3" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="B2" r:id="rId1" display="mailto:ahmad.fauzi@example.com" xr:uid="{4B90666F-B4DC-1D40-B23F-4994EB5457AC}"/>
+    <hyperlink ref="B2" r:id="rId1" xr:uid="{4B90666F-B4DC-1D40-B23F-4994EB5457AC}"/>
     <hyperlink ref="B3" r:id="rId2" xr:uid="{287C8E49-AD8F-6F42-A67A-401A81B9FCFC}"/>
     <hyperlink ref="B4" r:id="rId3" xr:uid="{5999E4BB-BE5E-A141-AB26-57D4AE28AF3D}"/>
   </hyperlinks>

</xml_diff>